<commit_message>
docs: simplify reviewer-facing language
</commit_message>
<xml_diff>
--- a/data/thesis_outputs/THESIS_OUTPUT_INDEX.xlsx
+++ b/data/thesis_outputs/THESIS_OUTPUT_INDEX.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="OUTPUT_INDEX" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OUTPUT_INDEX" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>canonical thesis and documented limitations</t>
+          <t>canonical thesis and execution notes</t>
         </is>
       </c>
     </row>

</xml_diff>